<commit_message>
Technical pack rebuilt: test strategy and cases, handover and architecture updates
</commit_message>
<xml_diff>
--- a/docs/technical/SalesVerse-2.0-Test-Cases.xlsx
+++ b/docs/technical/SalesVerse-2.0-Test-Cases.xlsx
@@ -798,7 +798,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2 October 2026, source commit af2fb05</t>
+          <t>2 October 2026, source commit d161514</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>As of 2 October 2026 (commit af2fb05); formulas count the Cases sheet, 'Catalogue' is the generator's count</t>
+          <t>As of 2 October 2026 (commit d161514); formulas count the Cases sheet, 'Catalogue' is the generator's count</t>
         </is>
       </c>
     </row>

</xml_diff>